<commit_message>
South Dakota: RHT series re-based to 26 contracts; 8 Rural Strong grants ($1,879,152) extracted, 5 hospital rows / $716,800
The Rural Strong rows sit INSIDE the $31.5M round and are asserted never to be added
to it. R/03bh's two now-stale SD verdicts removed; the rows match the file exactly.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MCsfF42a6CRzCkYZsYQXeg
</commit_message>
<xml_diff>
--- a/SD_rht_contracts.xlsx
+++ b/SD_rht_contracts.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="Contracts" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Reconciliation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Announced not published" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Announced rounds" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Outside the RHT series" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="355">
   <si>
     <t xml:space="preserve">state</t>
   </si>
@@ -136,6 +137,15 @@
     <t xml:space="preserve">description</t>
   </si>
   <si>
+    <t xml:space="preserve">award_pool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">round_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">first_seen_archive</t>
+  </si>
+  <si>
     <t xml:space="preserve">SD</t>
   </si>
   <si>
@@ -178,7 +188,7 @@
     <t xml:space="preserve">NON_HOSPITAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: commercial consultancy engaged through an RFP for services; named as the grant-programme management consultant in DOH's own release. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 26RHT00002, begun 2026-04-15. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: commercial consultancy engaged through an RFP for services; named as the grant-programme management consultant in DOH's own release. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 26RHT00002, begun 2026-04-15. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/26RHT00002.html</t>
@@ -211,6 +221,12 @@
     <t xml:space="preserve">Provide consultant services to SD Health Link to help manage the Digital Health Modernization and Technology Grant Program.</t>
   </si>
   <si>
+    <t xml:space="preserve">RHT series - programme administration, consulting, evaluation and workforce contracts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-28_open_sd_contract_search_RHT.html</t>
+  </si>
+  <si>
     <t xml:space="preserve">BUSINESS CONCEPTS &amp; APPS INC</t>
   </si>
   <si>
@@ -223,7 +239,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=26RHT00003</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: commercial consultancy engaged through an RFP for services; named as a project-management contractor in DOH's own release. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 26RHT00003, begun 2026-05-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: commercial consultancy engaged through an RFP for services; named as a project-management contractor in DOH's own release. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 26RHT00003, begun 2026-05-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/26RHT00003.html</t>
@@ -256,7 +272,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=26RHT00004</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: Community Health Worker Collaborative of South Dakota, a nonprofit; the register truncates the name. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 26RHT00004, begun 2026-05-07. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: Community Health Worker Collaborative of South Dakota, a nonprofit; the register truncates the name. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 26RHT00004, begun 2026-05-07. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/26RHT00004.html</t>
@@ -289,7 +305,7 @@
     <t xml:space="preserve">HIGH</t>
   </si>
   <si>
-    <t xml:space="preserve">Recipient name rule: name states a university or college. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 26RHT00006, begun 2026-05-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Recipient name rule: name states a university or college. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 26RHT00006, begun 2026-05-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/26RHT00006.html</t>
@@ -322,7 +338,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00001</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: South Dakota education service cooperative, a nonprofit. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00001, begun 2026-05-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: South Dakota education service cooperative, a nonprofit. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00001, begun 2026-05-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00001.html</t>
@@ -352,7 +368,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00005</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: national management consultancy engaged through an RFP for services. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00005, begun 2026-06-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: national management consultancy engaged through an RFP for services. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00005, begun 2026-06-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00005.html</t>
@@ -385,7 +401,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00007</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: actuarial and accounting firm engaged through an RFP for services. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00007, begun 2026-06-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: actuarial and accounting firm engaged through an RFP for services. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00007, begun 2026-06-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00007.html</t>
@@ -418,7 +434,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00008</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: Sioux Falls nonprofit senior services centre. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00008, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: Sioux Falls nonprofit senior services centre. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00008, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00008.html</t>
@@ -442,7 +458,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00009</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: South Dakota Foundation for Medical Care, the state's nonprofit quality improvement organisation. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00009, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: South Dakota Foundation for Medical Care, the state's nonprofit quality improvement organisation. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00009, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00009.html</t>
@@ -460,7 +476,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00010</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: South Dakota Foundation for Medical Care, the state's nonprofit quality improvement organisation. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00010, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: South Dakota Foundation for Medical Care, the state's nonprofit quality improvement organisation. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00010, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00010.html</t>
@@ -484,7 +500,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00011</t>
   </si>
   <si>
-    <t xml:space="preserve">Recipient name rule: name states a university or college. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00011, begun 2026-08-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Recipient name rule: name states a university or college. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00011, begun 2026-08-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00011.html</t>
@@ -511,7 +527,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00012</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: commercial health policy consultancy engaged through an RFP for services. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00012, begun 2026-06-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: commercial health policy consultancy engaged through an RFP for services. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00012, begun 2026-06-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00012.html</t>
@@ -541,7 +557,7 @@
     <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00013</t>
   </si>
   <si>
-    <t xml:space="preserve">Curated override: South Dakota Foundation for Medical Care, the state's nonprofit quality improvement organisation. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00013, begun 2026-07-17. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds, neither of which has been posted to this register.</t>
+    <t xml:space="preserve">Curated override: South Dakota Foundation for Medical Care, the state's nonprofit quality improvement organisation. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00013, begun 2026-07-17. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
   </si>
   <si>
     <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00013.html</t>
@@ -556,6 +572,354 @@
     <t xml:space="preserve">To establish regional EMS hubs that improve coordination, resource sharing, operational efficiency, and overall system performance across South Dakota.</t>
   </si>
   <si>
+    <t xml:space="preserve">SOUTH DAKOTA DOULAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECIPIENT_TYPE_INFERRED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient is named but the source does not state its organisational form; §8 settled fallback (session 10). §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00014, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00014.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALLBACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expand and strengthen the doula workforce in South Dakota through recruitment, training, certification, and workforce development activities.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-24_open_sd_contract_search_RHT.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD URBAN INDIAN HEALTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRIBAL_ORG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | NA | PIERRE, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a tribal entity. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00015, begun 2026-08-01. This is a RURAL STRONG GRANT -- the register's own description is 'Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program' -- one of the 28 grants ($31.5M) South Dakota announced on 2026-07-23 (KB0046839). It is INSIDE that round total and NEVER in addition to it: sd_year1_awardees.csv carries the round as one aggregate row whose round_amount ($31,500,000) already includes this contract. Tier 3, named recipient, primary source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00015.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RHT series - Rural Strong grants (subset of the 28-grant, $31.5M round of 2026-07-23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIVERSITY OF SOUTH DAKOTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | Contract with State or Local Government Agency (5-18D-21(8)) | VERMILLION, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a university or college. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00016, begun 2026-08-01. This is a RURAL STRONG GRANT -- the register's own description is 'Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program' -- one of the 28 grants ($31.5M) South Dakota announced on 2026-07-23 (KB0046839). It is INSIDE that round total and NEVER in addition to it: sd_year1_awardees.csv carries the round as one aggregate row whose round_amount ($31,500,000) already includes this contract. Tier 3, named recipient, primary source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00016.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERMILLION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPLETE HEALTH CENTER OF BH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | NA | RAPID CITY, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient is named but the source does not state its organisational form; §8 settled fallback (session 10). §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00017, begun 2026-08-01. This is a RURAL STRONG GRANT -- the register's own description is 'Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program' -- one of the 28 grants ($31.5M) South Dakota announced on 2026-07-23 (KB0046839). It is INSIDE that round total and NEVER in addition to it: sd_year1_awardees.csv carries the round as one aggregate row whose round_amount ($31,500,000) already includes this contract. Tier 3, named recipient, primary source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00017.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RAPID CITY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMMUNITY MEMORIAL HOSPITAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOSPITAL_OR_SYSTEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | NA | BURKE, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a hospital. §10.2 DIRECT: the named recipient is a hospital or hospital system and the state's award document names both the recipient and the amount. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00018, begun 2026-08-01. This is a RURAL STRONG GRANT -- the register's own description is 'Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program' -- one of the 28 grants ($31.5M) South Dakota announced on 2026-07-23 (KB0046839). It is INSIDE that round total and NEVER in addition to it: sd_year1_awardees.csv carries the round as one aggregate row whose round_amount ($31,500,000) already includes this contract. Tier 3, named recipient, primary source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00018.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BURKE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a university or college. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00019, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00019.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design, implement, host, and maintain a statewide education and training platform that expands access to high-quality, accredited training for all healthcare professionals in South Dakota, with a particular emphasis on supporting rural healthcare providers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | RFP (Linked) RFP Number: 26-09RHT-022 Solicitation Link: https://boa.sd.gov/central-services/procurement-management/ | STURGIS, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Curated override: South Dakota education service cooperative, a nonprofit. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00020, begun 2026-08-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00020.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFP (Linked) RFP Number: 26-09RHT-022 Solicitation Link: https://boa.sd.gov/central-services/procurement-management/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provide strategic leadership and operational support within the Office of Rural Health and Emergency Services in advancing rural healthcare transformation initiatives across the state.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a university or college. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00021, begun 2026-07-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00021.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAULKTON AREA MEDICAL CENTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | NA | FAULKTON, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">431301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMS Hospital Enrollments (archived data/evidence/SD/federal_records/2026-09-24/cms_hosp_enrollments_SD.json): ORGANIZATION NAME = the register's own string, city FAULKTON, CCN 431301, PART A PROVIDER - CRITICAL ACCESS HOSPITAL. Machine answer on the name: HOSPITAL_OR_SYSTEM/HIGH.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a medical center. §10.2 DIRECT: the named recipient is a hospital or hospital system and the state's award document names both the recipient and the amount. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00022, begun 2026-08-01. This is a RURAL STRONG GRANT -- the register's own description is 'Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program' -- one of the 28 grants ($31.5M) South Dakota announced on 2026-07-23 (KB0046839). It is INSIDE that round total and NEVER in addition to it: sd_year1_awardees.csv carries the round as one aggregate row whose round_amount ($31,500,000) already includes this contract. Tier 3, named recipient, primary source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00022.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAULKTON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHILIP HEALTH SERVICES INC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | NA | PHILIP, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">431319</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMS Hospital Enrollments (archived data/evidence/SD/federal_records/2026-09-24/cms_hosp_enrollments_SD.json): ORGANIZATION NAME = the register's own string, city PHILIP, CCN 431319, PART A PROVIDER - CRITICAL ACCESS HOSPITAL. Machine answer on the name: NONPROFIT_CBO/LOW.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient typed HOSPITAL_OR_SYSTEM on an ARCHIVED FEDERAL RECORD, not on its name: the register publishes no form, and CMS's Hospital Enrollments file carries this exact string in the same city (see recipient_type_source). MEDIUM, not HIGH: the match is on CMS's enrolment file, not an AHA/POS CCN reconciliation. §10.2 DIRECT: the named recipient is a hospital or hospital system and the state's award document names both the recipient and the amount. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00023, begun 2026-08-01. This is a RURAL STRONG GRANT -- the register's own description is 'Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program' -- one of the 28 grants ($31.5M) South Dakota announced on 2026-07-23 (KB0046839). It is INSIDE that round total and NEVER in addition to it: sd_year1_awardees.csv carries the round as one aggregate row whose round_amount ($31,500,000) already includes this contract. Tier 3, named recipient, primary source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00023.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FEDERAL_RECORD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHILIP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | NA | REDFIELD, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">431316</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CMS Hospital Enrollments (archived data/evidence/SD/federal_records/2026-09-24/cms_hosp_enrollments_SD.json): DOING BUSINESS AS NAME = the register's own string, city REDFIELD, CCN 431316, PART A PROVIDER - CRITICAL ACCESS HOSPITAL. Machine answer on the name: HOSPITAL_OR_SYSTEM/HIGH.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a hospital. §10.2 DIRECT: the named recipient is a hospital or hospital system and the state's award document names both the recipient and the amount. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00024, begun 2026-08-01. This is a RURAL STRONG GRANT -- the register's own description is 'Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program' -- one of the 28 grants ($31.5M) South Dakota announced on 2026-07-23 (KB0046839). It is INSIDE that round total and NEVER in addition to it: sd_year1_awardees.csv carries the round as one aggregate row whose round_amount ($31,500,000) already includes this contract. Tier 3, named recipient, primary source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00024.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REDFIELD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BENNETT COUNTY HOSPITAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | NA | MARTIN, SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a hospital. §10.2 DIRECT: the named recipient is a hospital or hospital system and the state's award document names both the recipient and the amount. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00025, begun 2026-08-01. This is a RURAL STRONG GRANT -- the register's own description is 'Implementation of a Rural Strong Grant as a part of the federal Rural Health Transformation Program' -- one of the 28 grants ($31.5M) South Dakota announced on 2026-07-23 (KB0046839). It is INSIDE that round total and NEVER in addition to it: sd_year1_awardees.csv carries the round as one aggregate row whose round_amount ($31,500,000) already includes this contract. Tier 3, named recipient, primary source.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00025.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARTIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENGINEERING SOLUTIONS INC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 - HEALTH | RFP (Linked) RFP Number: 27-09RHT-024 Solicitation Link: https://boa.sd.gov/central-services/procurement-management/ | WEST LINN, OR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota Open SD - Grants and Contracts register, contract 27RHT00026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://open.sd.gov/contractsDocShow.aspx?DocID=27RHT00026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recipient name rule: name states a technology vendor. §10.2 NON_HOSPITAL: the named recipient is not a hospital (§0.3a -- judged on the recipient, not the activity), and the source does not mention hospitals anywhere in the funded work. Source: South Dakota's Grants and Contracts register (SDCL 1-56-10 / 1-27-46), contract 27RHT00026, begun 2026-09-01. This is ADMINISTRATIVE RHTP spend and is NOT part of South Dakota's announced $31.5M (28 projects) or $90M (82 organisations) rounds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/evidence/SD/contract_details/27RHT00026.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFP (Linked) RFP Number: 27-09RHT-024 Solicitation Link: https://boa.sd.gov/central-services/procurement-management/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27RHT00026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WEST LINN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provide grant and administrative support for the Rural Health Transformation Project</t>
+  </si>
+  <si>
     <t xml:space="preserve">measure</t>
   </si>
   <si>
@@ -565,67 +929,91 @@
     <t xml:space="preserve">contracts extracted from the RHT series</t>
   </si>
   <si>
-    <t xml:space="preserve">13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">distinct vendors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">total extracted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,618,367.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">largest single contract</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,462,802.00</t>
+    <t xml:space="preserve">26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">distinct vendor strings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">total extracted (BOTH pools; never add to sd_year1_awardees.csv round totals)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9,223,177.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-- POOL 1: ADMINISTRATIVE --</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">administrative / programme contracts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">administrative total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7,344,025.00</t>
   </si>
   <si>
     <t xml:space="preserve">what these are</t>
   </si>
   <si>
-    <t xml:space="preserve">programme management, consulting, evaluation, workforce training</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-- NOT EXTRACTED, BECAUSE NOT PUBLISHED --</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Rural Strong round announced 2026-07-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$31,500,000 to 28 projects across 20 health systems</t>
+    <t xml:space="preserve">programme management, consulting, evaluation, workforce training, doula workforce, training platforms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-- POOL 2: RURAL STRONG GRANTS (Tier 3) --</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rural Strong grant contracts on the register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 of the 28 announced 2026-07-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rural Strong total on the register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,879,152.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rural Strong round total (KB0046839)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31,500,000.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">relationship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the register's contracts are INSIDE the round total; the round total already includes them</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rural Strong grants not yet on the register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 -- NAMED NOWHERE; their amount is stated by no source and is NOT computed here (§6.2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-- NOT ON THE REGISTER --</t>
   </si>
   <si>
     <t xml:space="preserve">Technology/data round announced 2026-08-19</t>
   </si>
   <si>
-    <t xml:space="preserve">$90,000,000 to 82 rural healthcare organizations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">either round found on open.sd.gov</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no</t>
-  </si>
-  <si>
-    <t xml:space="preserve">announcements archived</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no -- they are on news.sd.gov, refused at CONNECT (403)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">announced but unextracted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">121,500,000.00</t>
+    <t xml:space="preserve">$90,000,000 to 82 rural healthcare organizations -- no contract on open.sd.gov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RHTP contracts OUTSIDE the RHT series (not extracted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 -- 27SC091800 SD FOUNDATION FOR MEDICAL CARE $150,000; 26SC090058 BLACK HILLS SPECIAL SERVICES $ 45,000</t>
   </si>
   <si>
     <t xml:space="preserve">CMS Year 1 award for South Dakota</t>
@@ -640,13 +1028,16 @@
     <t xml:space="preserve">rows distributed_to_hospital = Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">0</t>
+    <t xml:space="preserve">5</t>
   </si>
   <si>
     <t xml:space="preserve">dollars distributed_to_hospital = Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">0.00</t>
+    <t xml:space="preserve">716,800.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">distinct hospitals among them</t>
   </si>
   <si>
     <t xml:space="preserve">round</t>
@@ -674,6 +1065,21 @@
   </si>
   <si>
     <t xml:space="preserve">82 rural healthcare organizations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">what</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27SC091800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">grant, begun 2026-05-01, CFDA 93.798; description is DOH's generic Rural Health Transformation paragraph -- RHTP money outside the series, a candidate for extraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26SC090058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contract, begun 2025-09-22 -- BEFORE the 2025-12-29 Notice of Award -- Professional Services under $50K; 'grant writing support for the Rural Health Transformation Program funding opportunity': APPLICATION support, not an award of RHTP money (§6.2 date test)</t>
   </si>
 </sst>
 </file>
@@ -1129,52 +1535,61 @@
       <c r="AN1" t="s">
         <v>39</v>
       </c>
+      <c r="AO1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D2" t="n">
         <v>1462802</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="L2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="M2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P2"/>
       <c r="Q2"/>
@@ -1182,107 +1597,114 @@
       <c r="S2"/>
       <c r="T2"/>
       <c r="U2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V2"/>
       <c r="W2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Z2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="AA2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="AB2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="AG2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="AH2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI2" s="1" t="n">
         <v>46127</v>
       </c>
       <c r="AJ2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL2" t="s">
         <v>63</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>40</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>60</v>
       </c>
       <c r="AM2"/>
       <c r="AN2" t="s">
-        <v>64</v>
+        <v>67</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP2"/>
+      <c r="AQ2" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D3" t="n">
         <v>250000</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K3" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P3"/>
       <c r="Q3"/>
@@ -1290,107 +1712,114 @@
       <c r="S3"/>
       <c r="T3"/>
       <c r="U3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V3"/>
       <c r="W3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="Z3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="AA3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="AB3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF3" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="AG3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="AH3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI3" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="AJ3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="AK3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL3" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="AM3"/>
       <c r="AN3" t="s">
-        <v>74</v>
+        <v>79</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP3"/>
+      <c r="AQ3" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D4" t="n">
         <v>399013</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="M4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P4"/>
       <c r="Q4"/>
@@ -1398,107 +1827,114 @@
       <c r="S4"/>
       <c r="T4"/>
       <c r="U4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V4"/>
       <c r="W4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="Z4" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="AA4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="AB4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AG4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="AH4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI4" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="AJ4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AK4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AM4"/>
       <c r="AN4" t="s">
-        <v>84</v>
+        <v>89</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP4"/>
+      <c r="AQ4" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D5" t="n">
         <v>225000</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K5" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="L5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="M5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P5"/>
       <c r="Q5"/>
@@ -1506,107 +1942,114 @@
       <c r="S5"/>
       <c r="T5"/>
       <c r="U5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="V5"/>
       <c r="W5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y5" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="Z5" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="AB5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE5" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="AF5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="AG5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="AH5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI5" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="AJ5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="AK5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="AM5"/>
       <c r="AN5" t="s">
-        <v>97</v>
+        <v>102</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP5"/>
+      <c r="AQ5" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D6" t="n">
         <v>503000</v>
       </c>
       <c r="E6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G6" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K6" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="L6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="M6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N6" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P6"/>
       <c r="Q6"/>
@@ -1614,107 +2057,114 @@
       <c r="S6"/>
       <c r="T6"/>
       <c r="U6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V6"/>
       <c r="W6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="Z6" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="AA6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="AB6" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF6" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="AG6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="AH6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI6" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="AJ6" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="AK6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL6" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="AM6"/>
       <c r="AN6" t="s">
-        <v>107</v>
+        <v>112</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP6"/>
+      <c r="AQ6" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D7" t="n">
         <v>567350</v>
       </c>
       <c r="E7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K7" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="L7" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="M7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P7"/>
       <c r="Q7"/>
@@ -1722,107 +2172,114 @@
       <c r="S7"/>
       <c r="T7"/>
       <c r="U7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="V7"/>
       <c r="W7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y7" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="Z7" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AA7" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AB7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF7" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="AG7" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="AH7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI7" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="AJ7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="AK7" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="AL7" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="AM7"/>
       <c r="AN7" t="s">
-        <v>118</v>
+        <v>123</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP7"/>
+      <c r="AQ7" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D8" t="n">
         <v>450000</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G8" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="L8" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P8"/>
       <c r="Q8"/>
@@ -1830,107 +2287,114 @@
       <c r="S8"/>
       <c r="T8"/>
       <c r="U8" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="V8"/>
       <c r="W8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="Z8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="AA8" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="AB8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF8" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="AG8" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="AH8" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI8" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="AJ8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="AK8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="AL8" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="AM8"/>
       <c r="AN8" t="s">
-        <v>129</v>
+        <v>134</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP8"/>
+      <c r="AQ8" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="D9" t="n">
         <v>226930</v>
       </c>
       <c r="E9" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K9" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="M9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P9"/>
       <c r="Q9"/>
@@ -1938,105 +2402,112 @@
       <c r="S9"/>
       <c r="T9"/>
       <c r="U9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V9"/>
       <c r="W9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y9" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="Z9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="AA9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="AB9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF9"/>
       <c r="AG9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="AH9" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI9" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="AJ9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AK9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL9"/>
       <c r="AM9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="AN9" t="s">
-        <v>138</v>
+        <v>143</v>
+      </c>
+      <c r="AO9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP9"/>
+      <c r="AQ9" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D10" t="n">
         <v>130571</v>
       </c>
       <c r="E10" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F10" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K10" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="L10" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="M10" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O10" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P10"/>
       <c r="Q10"/>
@@ -2044,105 +2515,112 @@
       <c r="S10"/>
       <c r="T10"/>
       <c r="U10" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V10"/>
       <c r="W10" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X10" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y10" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="Z10" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="AA10" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="AB10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF10"/>
       <c r="AG10" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="AH10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI10" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="AJ10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AK10" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL10"/>
       <c r="AM10" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="AN10" t="s">
-        <v>145</v>
+        <v>150</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP10"/>
+      <c r="AQ10" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D11" t="n">
         <v>170816</v>
       </c>
       <c r="E11" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F11" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G11" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="H11" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I11" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J11" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K11" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="L11" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="M11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P11"/>
       <c r="Q11"/>
@@ -2150,105 +2628,112 @@
       <c r="S11"/>
       <c r="T11"/>
       <c r="U11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V11"/>
       <c r="W11" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X11" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y11" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="Z11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="AA11" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="AB11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF11"/>
       <c r="AG11" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="AH11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI11" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="AJ11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AK11" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL11"/>
       <c r="AM11" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="AN11" t="s">
-        <v>151</v>
+        <v>156</v>
+      </c>
+      <c r="AO11" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP11"/>
+      <c r="AQ11" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D12" t="n">
         <v>88800</v>
       </c>
       <c r="E12" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F12" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G12" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I12" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J12" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K12" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="L12" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="M12" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N12" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O12" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P12"/>
       <c r="Q12"/>
@@ -2256,107 +2741,114 @@
       <c r="S12"/>
       <c r="T12"/>
       <c r="U12" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="V12"/>
       <c r="W12" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X12" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y12" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="Z12" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="AA12" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="AB12" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC12" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD12" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE12" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="AF12" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="AG12" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="AH12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI12" s="1" t="n">
         <v>46235</v>
       </c>
       <c r="AJ12" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AK12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL12" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="AM12"/>
       <c r="AN12" t="s">
-        <v>160</v>
+        <v>165</v>
+      </c>
+      <c r="AO12" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP12"/>
+      <c r="AQ12" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D13" t="n">
         <v>425000</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F13" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G13" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="H13" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I13" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J13" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K13" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="L13" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="M13" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O13" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P13"/>
       <c r="Q13"/>
@@ -2364,107 +2856,114 @@
       <c r="S13"/>
       <c r="T13"/>
       <c r="U13" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="V13"/>
       <c r="W13" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X13" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y13" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="Z13" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="AA13" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="AB13" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC13" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD13" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE13" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF13" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="AG13" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="AH13" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI13" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="AJ13" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="AK13" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="AL13" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="AM13"/>
       <c r="AN13" t="s">
-        <v>171</v>
+        <v>176</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP13"/>
+      <c r="AQ13" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D14" t="n">
         <v>719085</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G14" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="H14" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I14" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J14" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K14" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="L14" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M14" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N14" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O14" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P14"/>
       <c r="Q14"/>
@@ -2472,60 +2971,1578 @@
       <c r="S14"/>
       <c r="T14"/>
       <c r="U14" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="V14"/>
       <c r="W14" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="X14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="Y14" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="Z14" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="AA14" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="AB14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="AC14" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="AD14" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AE14" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="AF14" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="AG14" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="AH14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AI14" s="1" t="n">
         <v>46220</v>
       </c>
       <c r="AJ14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AK14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="AL14" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="AM14"/>
       <c r="AN14" t="s">
-        <v>179</v>
+        <v>184</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP14"/>
+      <c r="AQ14" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="s">
+        <v>185</v>
+      </c>
+      <c r="D15" t="n">
+        <v>133352</v>
+      </c>
+      <c r="E15" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" t="s">
+        <v>136</v>
+      </c>
+      <c r="H15" t="s">
+        <v>48</v>
+      </c>
+      <c r="I15" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K15" t="s">
+        <v>186</v>
+      </c>
+      <c r="L15" t="s">
+        <v>187</v>
+      </c>
+      <c r="M15" t="s">
+        <v>52</v>
+      </c>
+      <c r="N15" t="s">
+        <v>53</v>
+      </c>
+      <c r="O15" t="s">
+        <v>54</v>
+      </c>
+      <c r="P15"/>
+      <c r="Q15"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15"/>
+      <c r="U15" t="s">
+        <v>188</v>
+      </c>
+      <c r="V15" t="s">
+        <v>189</v>
+      </c>
+      <c r="W15" t="s">
+        <v>56</v>
+      </c>
+      <c r="X15" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>190</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>191</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>187</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>192</v>
+      </c>
+      <c r="AF15"/>
+      <c r="AG15" t="s">
+        <v>193</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI15" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK15" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL15"/>
+      <c r="AM15" t="s">
+        <v>142</v>
+      </c>
+      <c r="AN15" t="s">
+        <v>194</v>
+      </c>
+      <c r="AO15" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP15"/>
+      <c r="AQ15" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>196</v>
+      </c>
+      <c r="D16" t="n">
+        <v>467790</v>
+      </c>
+      <c r="E16" t="s">
+        <v>197</v>
+      </c>
+      <c r="F16" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" t="s">
+        <v>198</v>
+      </c>
+      <c r="H16" t="s">
+        <v>48</v>
+      </c>
+      <c r="I16" t="s">
+        <v>48</v>
+      </c>
+      <c r="J16" t="s">
+        <v>49</v>
+      </c>
+      <c r="K16" t="s">
+        <v>199</v>
+      </c>
+      <c r="L16" t="s">
+        <v>200</v>
+      </c>
+      <c r="M16" t="s">
+        <v>52</v>
+      </c>
+      <c r="N16" t="s">
+        <v>53</v>
+      </c>
+      <c r="O16" t="s">
+        <v>54</v>
+      </c>
+      <c r="P16"/>
+      <c r="Q16"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16"/>
+      <c r="U16" t="s">
+        <v>95</v>
+      </c>
+      <c r="V16"/>
+      <c r="W16" t="s">
+        <v>56</v>
+      </c>
+      <c r="X16" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>201</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>202</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>200</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF16"/>
+      <c r="AG16" t="s">
+        <v>203</v>
+      </c>
+      <c r="AH16" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI16" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>78</v>
+      </c>
+      <c r="AK16" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL16"/>
+      <c r="AM16" t="s">
+        <v>142</v>
+      </c>
+      <c r="AN16" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO16" t="s">
+        <v>205</v>
+      </c>
+      <c r="AP16" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ16" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>207</v>
+      </c>
+      <c r="D17" t="n">
+        <v>324000</v>
+      </c>
+      <c r="E17" t="s">
+        <v>91</v>
+      </c>
+      <c r="F17" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17" t="s">
+        <v>208</v>
+      </c>
+      <c r="H17" t="s">
+        <v>48</v>
+      </c>
+      <c r="I17" t="s">
+        <v>48</v>
+      </c>
+      <c r="J17" t="s">
+        <v>49</v>
+      </c>
+      <c r="K17" t="s">
+        <v>209</v>
+      </c>
+      <c r="L17" t="s">
+        <v>210</v>
+      </c>
+      <c r="M17" t="s">
+        <v>52</v>
+      </c>
+      <c r="N17" t="s">
+        <v>53</v>
+      </c>
+      <c r="O17" t="s">
+        <v>54</v>
+      </c>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17" t="s">
+        <v>95</v>
+      </c>
+      <c r="V17"/>
+      <c r="W17" t="s">
+        <v>56</v>
+      </c>
+      <c r="X17" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>211</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>212</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>210</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>99</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>213</v>
+      </c>
+      <c r="AH17" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI17" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>214</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>99</v>
+      </c>
+      <c r="AM17"/>
+      <c r="AN17" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO17" t="s">
+        <v>205</v>
+      </c>
+      <c r="AP17" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ17" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>215</v>
+      </c>
+      <c r="D18" t="n">
+        <v>370562</v>
+      </c>
+      <c r="E18" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" t="s">
+        <v>46</v>
+      </c>
+      <c r="G18" t="s">
+        <v>216</v>
+      </c>
+      <c r="H18" t="s">
+        <v>48</v>
+      </c>
+      <c r="I18" t="s">
+        <v>48</v>
+      </c>
+      <c r="J18" t="s">
+        <v>49</v>
+      </c>
+      <c r="K18" t="s">
+        <v>217</v>
+      </c>
+      <c r="L18" t="s">
+        <v>218</v>
+      </c>
+      <c r="M18" t="s">
+        <v>52</v>
+      </c>
+      <c r="N18" t="s">
+        <v>53</v>
+      </c>
+      <c r="O18" t="s">
+        <v>54</v>
+      </c>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18" t="s">
+        <v>188</v>
+      </c>
+      <c r="V18" t="s">
+        <v>189</v>
+      </c>
+      <c r="W18" t="s">
+        <v>56</v>
+      </c>
+      <c r="X18" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>219</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>220</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>218</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>192</v>
+      </c>
+      <c r="AF18"/>
+      <c r="AG18" t="s">
+        <v>221</v>
+      </c>
+      <c r="AH18" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI18" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ18" t="s">
+        <v>222</v>
+      </c>
+      <c r="AK18" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL18"/>
+      <c r="AM18" t="s">
+        <v>142</v>
+      </c>
+      <c r="AN18" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO18" t="s">
+        <v>205</v>
+      </c>
+      <c r="AP18" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ18" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>223</v>
+      </c>
+      <c r="D19" t="n">
+        <v>145500</v>
+      </c>
+      <c r="E19" t="s">
+        <v>224</v>
+      </c>
+      <c r="F19" t="s">
+        <v>48</v>
+      </c>
+      <c r="G19" t="s">
+        <v>225</v>
+      </c>
+      <c r="H19" t="s">
+        <v>48</v>
+      </c>
+      <c r="I19" t="s">
+        <v>48</v>
+      </c>
+      <c r="J19" t="s">
+        <v>49</v>
+      </c>
+      <c r="K19" t="s">
+        <v>226</v>
+      </c>
+      <c r="L19" t="s">
+        <v>227</v>
+      </c>
+      <c r="M19" t="s">
+        <v>52</v>
+      </c>
+      <c r="N19" t="s">
+        <v>53</v>
+      </c>
+      <c r="O19" t="s">
+        <v>54</v>
+      </c>
+      <c r="P19"/>
+      <c r="Q19"/>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19" t="s">
+        <v>95</v>
+      </c>
+      <c r="V19"/>
+      <c r="W19" t="s">
+        <v>228</v>
+      </c>
+      <c r="X19" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>229</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>230</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>227</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF19"/>
+      <c r="AG19" t="s">
+        <v>231</v>
+      </c>
+      <c r="AH19" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI19" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ19" t="s">
+        <v>232</v>
+      </c>
+      <c r="AK19" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL19"/>
+      <c r="AM19" t="s">
+        <v>142</v>
+      </c>
+      <c r="AN19" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO19" t="s">
+        <v>205</v>
+      </c>
+      <c r="AP19" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ19" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
+        <v>207</v>
+      </c>
+      <c r="D20" t="n">
+        <v>307228</v>
+      </c>
+      <c r="E20" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" t="s">
+        <v>46</v>
+      </c>
+      <c r="G20" t="s">
+        <v>208</v>
+      </c>
+      <c r="H20" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" t="s">
+        <v>48</v>
+      </c>
+      <c r="J20" t="s">
+        <v>49</v>
+      </c>
+      <c r="K20" t="s">
+        <v>233</v>
+      </c>
+      <c r="L20" t="s">
+        <v>234</v>
+      </c>
+      <c r="M20" t="s">
+        <v>52</v>
+      </c>
+      <c r="N20" t="s">
+        <v>53</v>
+      </c>
+      <c r="O20" t="s">
+        <v>54</v>
+      </c>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20" t="s">
+        <v>95</v>
+      </c>
+      <c r="V20"/>
+      <c r="W20" t="s">
+        <v>56</v>
+      </c>
+      <c r="X20" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>235</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>236</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>234</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>99</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>237</v>
+      </c>
+      <c r="AH20" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI20" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>214</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>99</v>
+      </c>
+      <c r="AM20"/>
+      <c r="AN20" t="s">
+        <v>238</v>
+      </c>
+      <c r="AO20" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP20"/>
+      <c r="AQ20" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>103</v>
+      </c>
+      <c r="D21" t="n">
+        <v>449402</v>
+      </c>
+      <c r="E21" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" t="s">
+        <v>46</v>
+      </c>
+      <c r="G21" t="s">
+        <v>239</v>
+      </c>
+      <c r="H21" t="s">
+        <v>48</v>
+      </c>
+      <c r="I21" t="s">
+        <v>48</v>
+      </c>
+      <c r="J21" t="s">
+        <v>49</v>
+      </c>
+      <c r="K21" t="s">
+        <v>240</v>
+      </c>
+      <c r="L21" t="s">
+        <v>241</v>
+      </c>
+      <c r="M21" t="s">
+        <v>52</v>
+      </c>
+      <c r="N21" t="s">
+        <v>53</v>
+      </c>
+      <c r="O21" t="s">
+        <v>54</v>
+      </c>
+      <c r="P21"/>
+      <c r="Q21"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+      <c r="U21" t="s">
+        <v>55</v>
+      </c>
+      <c r="V21"/>
+      <c r="W21" t="s">
+        <v>56</v>
+      </c>
+      <c r="X21" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>242</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>243</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>241</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>62</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>244</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>245</v>
+      </c>
+      <c r="AH21" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI21" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ21" t="s">
+        <v>111</v>
+      </c>
+      <c r="AK21" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL21" t="s">
+        <v>244</v>
+      </c>
+      <c r="AM21"/>
+      <c r="AN21" t="s">
+        <v>246</v>
+      </c>
+      <c r="AO21" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP21"/>
+      <c r="AQ21" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" t="n">
+        <v>185676</v>
+      </c>
+      <c r="E22" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" t="s">
+        <v>46</v>
+      </c>
+      <c r="G22" t="s">
+        <v>92</v>
+      </c>
+      <c r="H22" t="s">
+        <v>48</v>
+      </c>
+      <c r="I22" t="s">
+        <v>48</v>
+      </c>
+      <c r="J22" t="s">
+        <v>49</v>
+      </c>
+      <c r="K22" t="s">
+        <v>247</v>
+      </c>
+      <c r="L22" t="s">
+        <v>248</v>
+      </c>
+      <c r="M22" t="s">
+        <v>52</v>
+      </c>
+      <c r="N22" t="s">
+        <v>53</v>
+      </c>
+      <c r="O22" t="s">
+        <v>54</v>
+      </c>
+      <c r="P22"/>
+      <c r="Q22"/>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22"/>
+      <c r="U22" t="s">
+        <v>95</v>
+      </c>
+      <c r="V22"/>
+      <c r="W22" t="s">
+        <v>56</v>
+      </c>
+      <c r="X22" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>249</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>250</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>248</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>99</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>251</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI22" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="AJ22" t="s">
+        <v>101</v>
+      </c>
+      <c r="AK22" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL22" t="s">
+        <v>99</v>
+      </c>
+      <c r="AM22"/>
+      <c r="AN22" t="s">
+        <v>238</v>
+      </c>
+      <c r="AO22" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP22"/>
+      <c r="AQ22" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="s">
+        <v>252</v>
+      </c>
+      <c r="D23" t="n">
+        <v>38000</v>
+      </c>
+      <c r="E23" t="s">
+        <v>224</v>
+      </c>
+      <c r="F23" t="s">
+        <v>48</v>
+      </c>
+      <c r="G23" t="s">
+        <v>253</v>
+      </c>
+      <c r="H23" t="s">
+        <v>48</v>
+      </c>
+      <c r="I23" t="s">
+        <v>48</v>
+      </c>
+      <c r="J23" t="s">
+        <v>49</v>
+      </c>
+      <c r="K23" t="s">
+        <v>254</v>
+      </c>
+      <c r="L23" t="s">
+        <v>255</v>
+      </c>
+      <c r="M23" t="s">
+        <v>52</v>
+      </c>
+      <c r="N23" t="s">
+        <v>53</v>
+      </c>
+      <c r="O23" t="s">
+        <v>54</v>
+      </c>
+      <c r="P23" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23" t="s">
+        <v>257</v>
+      </c>
+      <c r="U23" t="s">
+        <v>95</v>
+      </c>
+      <c r="V23"/>
+      <c r="W23" t="s">
+        <v>228</v>
+      </c>
+      <c r="X23" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>258</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>259</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>255</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF23"/>
+      <c r="AG23" t="s">
+        <v>260</v>
+      </c>
+      <c r="AH23" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI23" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ23" t="s">
+        <v>261</v>
+      </c>
+      <c r="AK23" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL23"/>
+      <c r="AM23" t="s">
+        <v>142</v>
+      </c>
+      <c r="AN23" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO23" t="s">
+        <v>205</v>
+      </c>
+      <c r="AP23" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ23" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="s">
+        <v>262</v>
+      </c>
+      <c r="D24" t="n">
+        <v>181600</v>
+      </c>
+      <c r="E24" t="s">
+        <v>224</v>
+      </c>
+      <c r="F24" t="s">
+        <v>48</v>
+      </c>
+      <c r="G24" t="s">
+        <v>263</v>
+      </c>
+      <c r="H24" t="s">
+        <v>48</v>
+      </c>
+      <c r="I24" t="s">
+        <v>48</v>
+      </c>
+      <c r="J24" t="s">
+        <v>49</v>
+      </c>
+      <c r="K24" t="s">
+        <v>264</v>
+      </c>
+      <c r="L24" t="s">
+        <v>265</v>
+      </c>
+      <c r="M24" t="s">
+        <v>52</v>
+      </c>
+      <c r="N24" t="s">
+        <v>53</v>
+      </c>
+      <c r="O24" t="s">
+        <v>54</v>
+      </c>
+      <c r="P24" t="s">
+        <v>266</v>
+      </c>
+      <c r="Q24"/>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24" t="s">
+        <v>267</v>
+      </c>
+      <c r="U24" t="s">
+        <v>55</v>
+      </c>
+      <c r="V24"/>
+      <c r="W24" t="s">
+        <v>228</v>
+      </c>
+      <c r="X24" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>268</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>269</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>265</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>270</v>
+      </c>
+      <c r="AF24"/>
+      <c r="AG24" t="s">
+        <v>271</v>
+      </c>
+      <c r="AH24" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI24" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ24" t="s">
+        <v>272</v>
+      </c>
+      <c r="AK24" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL24"/>
+      <c r="AM24" t="s">
+        <v>142</v>
+      </c>
+      <c r="AN24" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO24" t="s">
+        <v>205</v>
+      </c>
+      <c r="AP24" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ24" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="s">
+        <v>223</v>
+      </c>
+      <c r="D25" t="n">
+        <v>103700</v>
+      </c>
+      <c r="E25" t="s">
+        <v>224</v>
+      </c>
+      <c r="F25" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" t="s">
+        <v>273</v>
+      </c>
+      <c r="H25" t="s">
+        <v>48</v>
+      </c>
+      <c r="I25" t="s">
+        <v>48</v>
+      </c>
+      <c r="J25" t="s">
+        <v>49</v>
+      </c>
+      <c r="K25" t="s">
+        <v>274</v>
+      </c>
+      <c r="L25" t="s">
+        <v>275</v>
+      </c>
+      <c r="M25" t="s">
+        <v>52</v>
+      </c>
+      <c r="N25" t="s">
+        <v>53</v>
+      </c>
+      <c r="O25" t="s">
+        <v>54</v>
+      </c>
+      <c r="P25" t="s">
+        <v>276</v>
+      </c>
+      <c r="Q25"/>
+      <c r="R25"/>
+      <c r="S25"/>
+      <c r="T25" t="s">
+        <v>277</v>
+      </c>
+      <c r="U25" t="s">
+        <v>95</v>
+      </c>
+      <c r="V25"/>
+      <c r="W25" t="s">
+        <v>228</v>
+      </c>
+      <c r="X25" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>278</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>279</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>275</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF25"/>
+      <c r="AG25" t="s">
+        <v>280</v>
+      </c>
+      <c r="AH25" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI25" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ25" t="s">
+        <v>281</v>
+      </c>
+      <c r="AK25" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL25"/>
+      <c r="AM25" t="s">
+        <v>142</v>
+      </c>
+      <c r="AN25" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO25" t="s">
+        <v>205</v>
+      </c>
+      <c r="AP25" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ25" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="s">
+        <v>282</v>
+      </c>
+      <c r="D26" t="n">
+        <v>248000</v>
+      </c>
+      <c r="E26" t="s">
+        <v>224</v>
+      </c>
+      <c r="F26" t="s">
+        <v>48</v>
+      </c>
+      <c r="G26" t="s">
+        <v>283</v>
+      </c>
+      <c r="H26" t="s">
+        <v>48</v>
+      </c>
+      <c r="I26" t="s">
+        <v>48</v>
+      </c>
+      <c r="J26" t="s">
+        <v>49</v>
+      </c>
+      <c r="K26" t="s">
+        <v>284</v>
+      </c>
+      <c r="L26" t="s">
+        <v>285</v>
+      </c>
+      <c r="M26" t="s">
+        <v>52</v>
+      </c>
+      <c r="N26" t="s">
+        <v>53</v>
+      </c>
+      <c r="O26" t="s">
+        <v>54</v>
+      </c>
+      <c r="P26"/>
+      <c r="Q26"/>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+      <c r="U26" t="s">
+        <v>95</v>
+      </c>
+      <c r="V26"/>
+      <c r="W26" t="s">
+        <v>228</v>
+      </c>
+      <c r="X26" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>286</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>287</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>285</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE26" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF26"/>
+      <c r="AG26" t="s">
+        <v>288</v>
+      </c>
+      <c r="AH26" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI26" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="AJ26" t="s">
+        <v>289</v>
+      </c>
+      <c r="AK26" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL26"/>
+      <c r="AM26" t="s">
+        <v>142</v>
+      </c>
+      <c r="AN26" t="s">
+        <v>204</v>
+      </c>
+      <c r="AO26" t="s">
+        <v>205</v>
+      </c>
+      <c r="AP26" t="s">
+        <v>206</v>
+      </c>
+      <c r="AQ26" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>43</v>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="s">
+        <v>290</v>
+      </c>
+      <c r="D27" t="n">
+        <v>650000</v>
+      </c>
+      <c r="E27" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" t="s">
+        <v>46</v>
+      </c>
+      <c r="G27" t="s">
+        <v>291</v>
+      </c>
+      <c r="H27" t="s">
+        <v>48</v>
+      </c>
+      <c r="I27" t="s">
+        <v>48</v>
+      </c>
+      <c r="J27" t="s">
+        <v>49</v>
+      </c>
+      <c r="K27" t="s">
+        <v>292</v>
+      </c>
+      <c r="L27" t="s">
+        <v>293</v>
+      </c>
+      <c r="M27" t="s">
+        <v>52</v>
+      </c>
+      <c r="N27" t="s">
+        <v>53</v>
+      </c>
+      <c r="O27" t="s">
+        <v>54</v>
+      </c>
+      <c r="P27"/>
+      <c r="Q27"/>
+      <c r="R27"/>
+      <c r="S27"/>
+      <c r="T27"/>
+      <c r="U27" t="s">
+        <v>55</v>
+      </c>
+      <c r="V27"/>
+      <c r="W27" t="s">
+        <v>56</v>
+      </c>
+      <c r="X27" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>294</v>
+      </c>
+      <c r="Z27" t="s">
+        <v>295</v>
+      </c>
+      <c r="AA27" t="s">
+        <v>293</v>
+      </c>
+      <c r="AB27" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC27" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD27" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE27" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF27" t="s">
+        <v>296</v>
+      </c>
+      <c r="AG27" t="s">
+        <v>297</v>
+      </c>
+      <c r="AH27" t="s">
+        <v>65</v>
+      </c>
+      <c r="AI27" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="AJ27" t="s">
+        <v>298</v>
+      </c>
+      <c r="AK27" t="s">
+        <v>299</v>
+      </c>
+      <c r="AL27" t="s">
+        <v>296</v>
+      </c>
+      <c r="AM27"/>
+      <c r="AN27" t="s">
+        <v>300</v>
+      </c>
+      <c r="AO27" t="s">
+        <v>68</v>
+      </c>
+      <c r="AP27"/>
+      <c r="AQ27" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -2541,130 +4558,178 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>180</v>
+        <v>301</v>
       </c>
       <c r="B1" t="s">
-        <v>181</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>182</v>
+        <v>303</v>
       </c>
       <c r="B2" t="s">
-        <v>183</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>184</v>
+        <v>305</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>186</v>
+        <v>307</v>
       </c>
       <c r="B4" t="s">
-        <v>187</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>188</v>
+        <v>309</v>
       </c>
       <c r="B5" t="s">
-        <v>189</v>
+        <v>310</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>190</v>
+        <v>311</v>
       </c>
       <c r="B6" t="s">
-        <v>191</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>192</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>194</v>
+        <v>315</v>
       </c>
       <c r="B8" t="s">
-        <v>195</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>196</v>
+        <v>317</v>
       </c>
       <c r="B9" t="s">
-        <v>197</v>
+        <v>310</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>198</v>
+        <v>318</v>
       </c>
       <c r="B10" t="s">
-        <v>199</v>
+        <v>319</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>200</v>
+        <v>320</v>
       </c>
       <c r="B11" t="s">
-        <v>201</v>
+        <v>321</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>202</v>
+        <v>322</v>
       </c>
       <c r="B12" t="s">
-        <v>203</v>
+        <v>323</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>204</v>
+        <v>324</v>
       </c>
       <c r="B13" t="s">
-        <v>205</v>
+        <v>325</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>206</v>
+        <v>326</v>
       </c>
       <c r="B14" t="s">
-        <v>193</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>207</v>
+        <v>328</v>
       </c>
       <c r="B15" t="s">
-        <v>208</v>
+        <v>310</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>209</v>
+        <v>329</v>
       </c>
       <c r="B16" t="s">
-        <v>210</v>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>331</v>
+      </c>
+      <c r="B17" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>333</v>
+      </c>
+      <c r="B18" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>335</v>
+      </c>
+      <c r="B19" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>336</v>
+      </c>
+      <c r="B20" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>338</v>
+      </c>
+      <c r="B21" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>340</v>
+      </c>
+      <c r="B22" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -2680,13 +4745,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>211</v>
+        <v>341</v>
       </c>
       <c r="B1" t="s">
-        <v>212</v>
+        <v>342</v>
       </c>
       <c r="C1" t="s">
-        <v>213</v>
+        <v>343</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
@@ -2694,13 +4759,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>344</v>
       </c>
       <c r="B2" t="s">
-        <v>215</v>
+        <v>345</v>
       </c>
       <c r="C2" t="s">
-        <v>216</v>
+        <v>346</v>
       </c>
       <c r="D2" t="n">
         <v>31500000</v>
@@ -2708,16 +4773,69 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>217</v>
+        <v>347</v>
       </c>
       <c r="B3" t="s">
-        <v>218</v>
+        <v>348</v>
       </c>
       <c r="C3" t="s">
-        <v>219</v>
+        <v>349</v>
       </c>
       <c r="D3" t="n">
         <v>90000000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D2" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>353</v>
+      </c>
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D3" t="s">
+        <v>354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>